<commit_message>
docs: GK-105 traz para o repositório a Sprint 0 da DoD e a aprovação do Plano de Qualidade
US: GK-105 [US-105] Planilhas da disciplina: DoD, Plano de Qualidade e Análise de Riscos

A versão do Drive tinha a coluna Sprint 0 da DoD preenchida (13 Sim, 1 Não e
9 N/A, 93%) e o Plano de Qualidade aprovado por Wagner Tiburcio; a cópia do
repositório ainda não tinha esses valores. Agora as duas versões são iguais.
</commit_message>
<xml_diff>
--- a/docs/DoD-Sprint-e-Release.xlsx
+++ b/docs/DoD-Sprint-e-Release.xlsx
@@ -1051,7 +1051,11 @@
           <t>PO</t>
         </is>
       </c>
-      <c r="D5" s="5" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
@@ -1080,7 +1084,11 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
@@ -1113,7 +1121,11 @@
           <t>PO</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
@@ -1138,7 +1150,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n"/>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
@@ -1163,7 +1179,11 @@
           <t>PO</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E9" s="5" t="n"/>
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
@@ -1207,7 +1227,11 @@
           <t>DevOps</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -1244,7 +1268,11 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n"/>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -1281,7 +1309,11 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -1318,7 +1350,11 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
@@ -1362,7 +1398,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D16" s="5" t="n"/>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
@@ -1387,7 +1427,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D17" s="5" t="n"/>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -1424,7 +1468,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D18" s="5" t="n"/>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="n"/>
@@ -1449,7 +1497,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D19" s="5" t="n"/>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="n"/>
@@ -1474,7 +1526,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D20" s="5" t="n"/>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="5" t="n"/>
@@ -1499,7 +1555,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D21" s="5" t="n"/>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
       <c r="G21" s="5" t="n"/>
@@ -1543,7 +1603,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D23" s="5" t="n"/>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
@@ -1568,7 +1632,11 @@
           <t>PO</t>
         </is>
       </c>
-      <c r="D24" s="5" t="n"/>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="5" t="n"/>
@@ -1593,7 +1661,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D25" s="5" t="n"/>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E25" s="5" t="n"/>
       <c r="F25" s="5" t="n"/>
       <c r="G25" s="5" t="n"/>
@@ -1618,7 +1690,11 @@
           <t>PO</t>
         </is>
       </c>
-      <c r="D26" s="5" t="n"/>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
       <c r="G26" s="5" t="n"/>
@@ -1662,7 +1738,11 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="D28" s="5" t="n"/>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E28" s="5" t="n"/>
       <c r="F28" s="5" t="n"/>
       <c r="G28" s="5" t="n"/>
@@ -1695,7 +1775,11 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="D29" s="5" t="n"/>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -1728,7 +1812,11 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="D30" s="5" t="n"/>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E30" s="5" t="n"/>
       <c r="F30" s="5" t="n"/>
       <c r="G30" s="5" t="n"/>
@@ -1753,7 +1841,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D31" s="5" t="n"/>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E31" s="5" t="n"/>
       <c r="F31" s="5" t="n"/>
       <c r="G31" s="5" t="n"/>

</xml_diff>

<commit_message>
docs: GK-105 prepara o fechamento da Release 1 e os papéis da Release 2
US: GK-105 [US-105] Planilhas da disciplina: DoD, Plano de Qualidade e Análise de Riscos

- Plano de Teste v1.1: status dos 30 casos a partir do CI da main
  (30/30 aprovados) e métricas da Sprint 1; Q-08 em 100%.
- Release Notes e Relatório de Qualidade R1 preenchidos com os dados
  de 28/10; novos Relatório de Métricas (velocity, burndown) e
  Relatório do Pipeline.
- Ata da Review com pauta e dados; presença, demonstração e feedback
  ficam para a reunião de 29/10.
- README com os papéis da Release 2 (Pedro SM, Wagner PO e DevOps,
  Rodrigo QA) e a passagem de bastão.
- DoD e Plano de Qualidade atualizados com o aceite do PO, o backlog
  repriorizado, a DoR da Release 2 e os relatórios da release.
</commit_message>
<xml_diff>
--- a/docs/DoD-Sprint-e-Release.xlsx
+++ b/docs/DoD-Sprint-e-Release.xlsx
@@ -1154,7 +1154,11 @@
       <c r="J8" s="5" t="n"/>
       <c r="K8" s="5" t="n"/>
       <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Review marcada para 29/10/2026; demonstração de cadastro, login, catálogo e detalhe. Marcar depois da reunião.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="22.04999923706055" customHeight="1" s="10">
       <c r="A9" s="5" t="n">
@@ -1175,17 +1179,25 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="E9" s="5" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n"/>
       <c r="I9" s="5" t="n"/>
       <c r="J9" s="5" t="n"/>
       <c r="K9" s="5" t="n"/>
-      <c r="L9" s="3" t="n"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>https://pedrolucas0721.atlassian.net/browse/GK-9</t>
+        </is>
+      </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>Aceite do PO e QA registrados em cada card só em GK-7, GK-8, GK-105 e GK-106 (28/10/2026). GK-9, GK-10, GK-57, GK-58 e GK-63 têm apenas o aceite geral do PO registrado na GK-61; registrar o aceite em cada card na Review de 29/10.</t>
+          <t>Aceite do PO registrado em cada card em 28/10/2026: GK-7, GK-8, GK-9, GK-10, GK-57, GK-58, GK-63 (e GK-105, GK-106). GK-61 é aceita na Review.</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1667,11 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E23" s="5" t="n"/>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
       <c r="H23" s="5" t="n"/>
@@ -1664,12 +1680,12 @@
       <c r="K23" s="5" t="n"/>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>docs/sprints/Acompanhamento-e-Resultados-Sprint-1.docx; GK-97</t>
+          <t>docs/releases/Relatorio-de-Metricas-R1.docx; docs/sprints/Acompanhamento-e-Resultados-Sprint-1.docx</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>Métricas de 28/10/2026 (antes da Review): 28 pontos planejados, 27 concluídos no Jira (96%), 1 Em revisão (GK-61). Velocity e burndown finais no fechamento da sprint em 29/10.</t>
+          <t>Velocity e burndown da Sprint 1 no Relatório de Métricas R1: 27 de 28 pontos em 28/10/2026; atualizar a GK-61 (1 ponto) no fechamento de 29/10.</t>
         </is>
       </c>
     </row>
@@ -1692,15 +1708,27 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="E24" s="5" t="n"/>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="5" t="n"/>
       <c r="H24" s="5" t="n"/>
       <c r="I24" s="5" t="n"/>
       <c r="J24" s="5" t="n"/>
       <c r="K24" s="5" t="n"/>
-      <c r="L24" s="3" t="n"/>
-      <c r="M24" s="3" t="n"/>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>https://pedrolucas0721.atlassian.net/browse/GK-3</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>Backlog da Release 2 repriorizado pelo PO em 28/10/2026 pela ordem de dependência (GK-11, GK-12, GK-15, GK-14, GK-16, GK-13, GK-48, GK-68), com proposta para a Sprint 2.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="22.04999923706055" customHeight="1" s="10">
       <c r="A25" s="5" t="n">
@@ -1758,15 +1786,27 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="E26" s="5" t="n"/>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="F26" s="5" t="n"/>
       <c r="G26" s="5" t="n"/>
       <c r="H26" s="5" t="n"/>
       <c r="I26" s="5" t="n"/>
       <c r="J26" s="5" t="n"/>
       <c r="K26" s="5" t="n"/>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>https://pedrolucas0721.atlassian.net/browse/GK-3</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>GK-11 a GK-16 com Gherkin, story points, prioridade, dependências e DoR completa em 28/10/2026. RNFs GK-46, GK-47 e GK-48 estimados no Planning Poker da Sprint 2.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
@@ -1933,7 +1973,11 @@
       <c r="J31" s="5" t="n"/>
       <c r="K31" s="5" t="n"/>
       <c r="L31" s="3" t="n"/>
-      <c r="M31" s="3" t="n"/>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>Conferir o dashboard GameKeys - Relatórios e as datas da Sprint 1 no Jira na Review de 29/10.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="4" t="inlineStr">
@@ -2146,7 +2190,11 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Demonstração na Review de 29/10/2026, no ambiente de desenvolvimento documentado. Marcar depois da reunião.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22.04999923706055" customHeight="1" s="10">
       <c r="A6" s="5" t="n">
@@ -2293,7 +2341,11 @@
           <t>PO</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
@@ -2304,7 +2356,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Rascunho; completar na Review de 29/10.</t>
+          <t>Entregas, RNFs, itens fora, problemas conhecidos, números e próxima release preenchidos em 28/10/2026.</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2374,11 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n"/>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
@@ -2333,7 +2389,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Modelo pronto; preencher com os resultados R1 do Plano de Qualidade.</t>
+          <t>15 metas com Resultado R1 e Atendeu?, 30 de 30 casos executados, bugs, DoD dos itens, regressão e ações de melhoria (28/10/2026).</t>
         </is>
       </c>
     </row>
@@ -2351,12 +2407,24 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>docs/releases/Relatorio-de-Metricas-R1.docx</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Velocity, burndown da Sprint 1, impedimentos e indicadores de processo (28/10/2026).</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="22.04999923706055" customHeight="1" s="10">
       <c r="A14" s="5" t="n">
@@ -2372,12 +2440,24 @@
           <t>DevOps</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>docs/releases/Relatorio-do-Pipeline-R1.docx</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Etapas do CI, 32 de 32 execuções verdes na main, duração e mudanças da Release 1 (28/10/2026).</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="31.95000076293945" customHeight="1" s="10">
       <c r="A15" s="5" t="n">
@@ -2398,7 +2478,11 @@
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
       <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Seção 8 da Ata da Retrospectiva, preenchida na reunião de 29/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
@@ -2429,7 +2513,11 @@
           <t>PO</t>
         </is>
       </c>
-      <c r="D17" s="5" t="n"/>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="inlineStr">
@@ -2437,8 +2525,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>https://pedrolucas0721.atlassian.net/browse/GK-3</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Release 2 repriorizada pelo PO em 28/10/2026 pela ordem de dependência; ajustar com o feedback da Review, se houver.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="22.04999923706055" customHeight="1" s="10">
       <c r="A18" s="5" t="n">
@@ -2454,7 +2550,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D18" s="5" t="n"/>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="inlineStr">
@@ -2462,8 +2562,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/PedroLuvaz/gamekeys-uepb-2026-2#equipe</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Release 2: Pedro SM, Wagner PO e DevOps, Rodrigo QA.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="22.04999923706055" customHeight="1" s="10">
       <c r="A19" s="5" t="n">
@@ -2479,7 +2587,11 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="D19" s="5" t="n"/>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="inlineStr">
@@ -2487,8 +2599,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>README.md, seção Equipe</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Passagem de bastão por papel registrada no README (o que cada um recebe e o que fica em aberto).</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="22.04999923706055" customHeight="1" s="10">
       <c r="A20" s="5" t="n">
@@ -2509,7 +2629,11 @@
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="5" t="n"/>
       <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Cada integrante preenche a avaliação entre pares no fechamento da Release 1.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="22.04999923706055" customHeight="1" s="10">
       <c r="A21" s="5" t="n">
@@ -2881,14 +3005,18 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="D33" s="5" t="n"/>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="E33" s="5" t="n"/>
       <c r="F33" s="5" t="n"/>
       <c r="G33" s="5" t="n"/>
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Resultado R1 dos 15 itens registrado no Relatório de Qualidade R1 e no Plano de Qualidade em 28/10/2026; falta a coluna Atendeu? e a execução formal dos casos pelo QA.</t>
+          <t>Resultado R1 e Atendeu? das 15 metas no Relatório de Qualidade R1 e no Plano de Qualidade (28/10/2026): 12 de 13 aplicáveis atendidas; Q-11 não atendida.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: GK-38 registra a aprovação do acordo da DoD pela equipe na Planning
US: GK-38 Definir Definition of Ready e Definition of Done
Documento: GK-105 [US-105] Planilhas da disciplina

O histórico do acordo dizia "A confirmar pela equipe na Planning da Sprint 1".
Agora registra a aprovação de Pedro, Wagner e Rodrigo na Planning de
20/10/2026, e as assinaturas de ciência ganham a data do acordo.
</commit_message>
<xml_diff>
--- a/docs/DoD-Sprint-e-Release.xlsx
+++ b/docs/DoD-Sprint-e-Release.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acordo da equipe" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DoD da Sprint" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DoD da Release" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Acordo da equipe" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="DoD da Sprint" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DoD da Release" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -797,7 +798,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>A confirmar pela equipe na Planning da Sprint 1</t>
+          <t>Equipe (Pedro, Wagner e Rodrigo) na Planning da Sprint 1, em 20/10/2026</t>
         </is>
       </c>
     </row>
@@ -839,7 +840,7 @@
     <row r="29">
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Pedro Lucas Vaz de Andrade - PO e DevOps (Release 1)</t>
+          <t>Pedro Lucas Vaz de Andrade - PO e DevOps (Release 1) - de acordo em 20/10/2026</t>
         </is>
       </c>
       <c r="C29" s="15" t="n"/>
@@ -850,7 +851,7 @@
     <row r="30">
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Wagner Tiburcio da Silva Junior - QA (Release 1)</t>
+          <t>Wagner Tiburcio da Silva Junior - QA (Release 1) - de acordo em 20/10/2026</t>
         </is>
       </c>
       <c r="C30" s="15" t="n"/>
@@ -861,7 +862,7 @@
     <row r="31">
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Rodrigo Almeida Gomes - Scrum Master (Release 1)</t>
+          <t>Rodrigo Almeida Gomes - Scrum Master (Release 1) - de acordo em 20/10/2026</t>
         </is>
       </c>
       <c r="C31" s="15" t="n"/>

</xml_diff>

<commit_message>
docs: GK-105 prepara a DoD e o Plano de Qualidade para os papéis da Release 2
US: GK-105 [US-105] Planilhas da disciplina: DoD, Plano de Qualidade e Análise de Riscos

- DoD: Pedro passa a ser o SM responsável pela manutenção do acordo e
  entram as assinaturas da Release 2 (Pedro SM, Wagner PO e DevOps,
  Rodrigo QA), com o "de acordo" pendente para a Planning de 03/11.
- Plano de Qualidade v1.1: coluna Responsável de Q-01 a Q-15 com os
  papéis da Release 2, registrada na aba Revisões. Metas e Resultado R1
  sem mudança.
- Análise de Riscos sem mudança: cada risco segue com o integrante que
  o identificou.
</commit_message>
<xml_diff>
--- a/docs/DoD-Sprint-e-Release.xlsx
+++ b/docs/DoD-Sprint-e-Release.xlsx
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F32"/>
+  <dimension ref="B1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.39999961853027"/>
   <cols>
     <col width="3" customWidth="1" style="10" min="1" max="1"/>
@@ -670,7 +670,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Rodrigo Almeida Gomes</t>
+          <t>Pedro Lucas Vaz de Andrade (Release 2; Rodrigo Almeida Gomes na Release 1)</t>
         </is>
       </c>
       <c r="D8" s="15" t="n"/>
@@ -859,7 +859,7 @@
       <c r="E30" s="15" t="n"/>
       <c r="F30" s="16" t="n"/>
     </row>
-    <row r="31">
+    <row r="31" s="10">
       <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Rodrigo Almeida Gomes - Scrum Master (Release 1) - de acordo em 20/10/2026</t>
@@ -870,15 +870,41 @@
       <c r="E31" s="15" t="n"/>
       <c r="F31" s="16" t="n"/>
     </row>
-    <row r="32">
-      <c r="B32" s="8" t="inlineStr"/>
+    <row r="32" s="10">
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Pedro Lucas Vaz de Andrade - Scrum Master (Release 2) - de acordo pendente, Planning da Sprint 2 em 03/11/2026</t>
+        </is>
+      </c>
       <c r="C32" s="15" t="n"/>
       <c r="D32" s="15" t="n"/>
       <c r="E32" s="15" t="n"/>
       <c r="F32" s="16" t="n"/>
     </row>
+    <row r="33" s="10">
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Wagner Tiburcio da Silva Junior - PO e DevOps (Release 2) - de acordo pendente, Planning da Sprint 2 em 03/11/2026</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="15" t="n"/>
+      <c r="E33" s="15" t="n"/>
+      <c r="F33" s="16" t="n"/>
+    </row>
+    <row r="34" s="10">
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Rodrigo Almeida Gomes - QA (Release 2) - de acordo pendente, Planning da Sprint 2 em 03/11/2026</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="16" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="22">
     <mergeCell ref="C8:F8"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="C7:F7"/>
@@ -893,11 +919,13 @@
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B34:F34"/>
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="B19:F19"/>
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="C9:F9"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B33:F33"/>
     <mergeCell ref="B32:F32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>